<commit_message>
Daily sync: 2026-10-11 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3328,807 +3328,1725 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>daily-20</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>Buccaneers +8.5 (-105)</t>
-        </is>
-      </c>
-      <c r="D59" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="6" t="inlineStr"/>
-      <c r="F59" s="6" t="inlineStr"/>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Buccaneers +8.5 (-105) ✓</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Over 47.5 (-110) ✗</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>White Sox ML (+102) ✗</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Bruins ML (+100) ✓</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Hurricanes -1.5 (-132) ✓</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Blues ML (-160) ✗</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Under 49.5 (-105) ✗</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>BetMGM</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Over 7.5 (-104) ✓</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Golden Knights ML (-162) ✓</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="5" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Avalanche -1.5 (+104) ✓</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr"/>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr"/>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Under 6.5 (-130) ✗</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Under 6.5 (-120) ✗</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Sabres ML (-106) ✗</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Liberty -13.5 (-105) ✓</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="4" t="inlineStr"/>
+      <c r="F72" s="4" t="inlineStr"/>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="5" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>South Alabama +2.5 (-108) ✓</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>BetRivers</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="5" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>WKU -1.5 (-110) ✓</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr"/>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>consensus (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="5" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Mammoth ML (-120) ✗</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Wild +1.5 (-205) ✓</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="4" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr"/>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr"/>
+      <c r="L76" s="5" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Buccaneers ML (+360) ✓</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="5" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Under 6.5 (-110) ✗</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>consensus (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Dream ML (+136) ✓</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Valkyries ML (+155) ✓</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr"/>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr"/>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>wunderdog consensus (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Under 42.5 (-102) ✓</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="5" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Florida State +3.5 (-108) ✗</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Under 43.5 (-115) ✓</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="5" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Dream +3.5 (-110) ✓</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="4" t="inlineStr"/>
+      <c r="F84" s="4" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="5" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Under 41.5 (-115) ✗</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Utah State -5.5 (-108) ✗</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Under 48.5 (-110) ✓</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="5" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Valkyries +4 (-110) ✓</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="4" t="inlineStr"/>
+      <c r="F88" s="4" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr"/>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>wunderdog consensus (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="5" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Florida State ML (+150) ✗</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Rangers ML (+120) ✗</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Washington -2.5 (-115) ✗</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Ducks ML (+110) ✓</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="4" t="inlineStr"/>
+      <c r="F92" s="4" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr"/>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Penguins ML (+103) ✗</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Over 59.5 (-105) ✓</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="4" t="inlineStr"/>
+      <c r="F94" s="4" t="inlineStr"/>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr"/>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="5" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Over 172.5 (-105) ✗</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>wunderdog consensus (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Kraken ML (+120) ✓</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="4" t="inlineStr"/>
+      <c r="F96" s="4" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="5" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Blue Jackets ML (-121) ✓</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="4" t="inlineStr"/>
+      <c r="F97" s="4" t="inlineStr"/>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel (verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="5" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Jets ML (-125) ✗</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Under 39.5 (-110) ✗
+Alabama -1.5 (-112) ✗
+Lightning ML (-164) ✓
+North Dakota State -3.5 (-110) ✗
+Missouri -3.5 (-105) ✓
+Georgia +1.5 (-110) ✓
+Under 51.5 (-110) ✓
+Panthers ML (-134) ✗
+Devils ML (-275) ✓
+Kansas State -2.5 (-110) ✗
+Navy -1.5 (-110) ✓
+Fresno State +7 (-110)
+Guardians ML (-135) ✓
+Avalanche ML (-215) ✗
+Hurricanes ML (-250) ✓
+Sabres ML (-110) ✗
+Indiana -7.5 (-110) ✗
+USC +1.5 (-110) ✓
+South Carolina +12.5 (-110) ✓
+Over 7 (-120) ✗</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E99" s="4" t="inlineStr"/>
+      <c r="F99" s="4" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr"/>
+      <c r="L99" s="5" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>Browns +2.5 (-110)
+Vikings -2.5 (+100)
+Under 46.5 (-118)
+Browns ML (+114)
+Over 43.5 (-108)
+Eagles +7.5 (+100)
+Dolphins +7 (-110)
+Giants +3.5 (-108)
+Titans +7 (-112)
+Over 41.5 (-105)
+Over 54.5 (-105)
+Under 41.5 (-108)
+Under 43.5 (-112)
+Over 45.5 (-115)
+Under 43.5 (-110)
+Over 45.5 (-105)
+49ers +3 (-105)
+Chargers +3.5 (-112)
+Under 41.5 (-115)
+Colts +2.5 (+100)</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E100" s="6" t="inlineStr"/>
+      <c r="F100" s="6" t="inlineStr"/>
+      <c r="G100" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr"/>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="H100" s="6" t="inlineStr"/>
+      <c r="I100" s="6" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K59" s="6" t="inlineStr"/>
-      <c r="L59" s="7" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="inlineStr">
-        <is>
-          <t>Over 47.5 (-110)</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="6" t="inlineStr"/>
-      <c r="F60" s="6" t="inlineStr"/>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr"/>
-      <c r="I60" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings</t>
-        </is>
-      </c>
-      <c r="J60" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K60" s="6" t="inlineStr"/>
-      <c r="L60" s="7" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>White Sox ML (+102)</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="6" t="inlineStr"/>
-      <c r="F61" s="6" t="inlineStr"/>
-      <c r="G61" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr"/>
-      <c r="I61" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J61" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K61" s="6" t="inlineStr"/>
-      <c r="L61" s="7" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>Bruins ML (+100)</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="6" t="inlineStr"/>
-      <c r="F62" s="6" t="inlineStr"/>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr"/>
-      <c r="I62" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J62" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K62" s="6" t="inlineStr"/>
-      <c r="L62" s="7" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>Hurricanes -1.5 (-132)</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="6" t="inlineStr"/>
-      <c r="F63" s="6" t="inlineStr"/>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr"/>
-      <c r="I63" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J63" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K63" s="6" t="inlineStr"/>
-      <c r="L63" s="7" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>Blues ML (-160)</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="6" t="inlineStr"/>
-      <c r="F64" s="6" t="inlineStr"/>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr"/>
-      <c r="I64" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J64" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K64" s="6" t="inlineStr"/>
-      <c r="L64" s="7" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>Under 49.5 (-105)</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="6" t="inlineStr"/>
-      <c r="F65" s="6" t="inlineStr"/>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr"/>
-      <c r="I65" s="6" t="inlineStr">
-        <is>
-          <t>BetMGM</t>
-        </is>
-      </c>
-      <c r="J65" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K65" s="6" t="inlineStr"/>
-      <c r="L65" s="7" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>Over 7.5 (-104)</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="6" t="inlineStr"/>
-      <c r="F66" s="6" t="inlineStr"/>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr"/>
-      <c r="I66" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J66" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K66" s="6" t="inlineStr"/>
-      <c r="L66" s="7" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>Golden Knights ML (-162)</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="6" t="inlineStr"/>
-      <c r="F67" s="6" t="inlineStr"/>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr"/>
-      <c r="I67" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J67" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K67" s="6" t="inlineStr"/>
-      <c r="L67" s="7" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>Avalanche -1.5 (+104)</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="6" t="inlineStr"/>
-      <c r="F68" s="6" t="inlineStr"/>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="inlineStr"/>
-      <c r="I68" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J68" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K68" s="6" t="inlineStr"/>
-      <c r="L68" s="7" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>Under 6.5 (-130)</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="6" t="inlineStr"/>
-      <c r="F69" s="6" t="inlineStr"/>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr"/>
-      <c r="I69" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J69" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K69" s="6" t="inlineStr"/>
-      <c r="L69" s="7" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>Under 6.5 (-120)</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="6" t="inlineStr"/>
-      <c r="F70" s="6" t="inlineStr"/>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr"/>
-      <c r="I70" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J70" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K70" s="6" t="inlineStr"/>
-      <c r="L70" s="7" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="inlineStr">
-        <is>
-          <t>Sabres ML (-106)</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="6" t="inlineStr"/>
-      <c r="F71" s="6" t="inlineStr"/>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr"/>
-      <c r="I71" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J71" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K71" s="6" t="inlineStr"/>
-      <c r="L71" s="7" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>Liberty -13.5 (-105)</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="6" t="inlineStr"/>
-      <c r="F72" s="6" t="inlineStr"/>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H72" s="6" t="inlineStr"/>
-      <c r="I72" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K72" s="6" t="inlineStr"/>
-      <c r="L72" s="7" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>South Alabama +2.5 (-108)</t>
-        </is>
-      </c>
-      <c r="D73" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" s="6" t="inlineStr"/>
-      <c r="F73" s="6" t="inlineStr"/>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="inlineStr"/>
-      <c r="I73" s="6" t="inlineStr">
-        <is>
-          <t>BetRivers</t>
-        </is>
-      </c>
-      <c r="J73" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K73" s="6" t="inlineStr"/>
-      <c r="L73" s="7" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr">
-        <is>
-          <t>WKU -1.5 (-110)</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E74" s="6" t="inlineStr"/>
-      <c r="F74" s="6" t="inlineStr"/>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H74" s="6" t="inlineStr"/>
-      <c r="I74" s="6" t="inlineStr">
-        <is>
-          <t>consensus (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J74" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K74" s="6" t="inlineStr"/>
-      <c r="L74" s="7" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>Mammoth ML (-120)</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E75" s="6" t="inlineStr"/>
-      <c r="F75" s="6" t="inlineStr"/>
-      <c r="G75" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H75" s="6" t="inlineStr"/>
-      <c r="I75" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J75" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K75" s="6" t="inlineStr"/>
-      <c r="L75" s="7" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="inlineStr">
-        <is>
-          <t>Wild +1.5 (-205)</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="6" t="inlineStr"/>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H76" s="6" t="inlineStr"/>
-      <c r="I76" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J76" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K76" s="6" t="inlineStr"/>
-      <c r="L76" s="7" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C77" s="7" t="inlineStr">
-        <is>
-          <t>Buccaneers ML (+360)</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="6" t="inlineStr"/>
-      <c r="F77" s="6" t="inlineStr"/>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr"/>
-      <c r="I77" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings</t>
-        </is>
-      </c>
-      <c r="J77" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K77" s="6" t="inlineStr"/>
-      <c r="L77" s="7" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>Under 6.5 (-110)</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="6" t="inlineStr"/>
-      <c r="G78" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H78" s="6" t="inlineStr"/>
-      <c r="I78" s="6" t="inlineStr">
-        <is>
-          <t>consensus (verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J78" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K78" s="6" t="inlineStr"/>
-      <c r="L78" s="7" t="inlineStr"/>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
+      <c r="L100" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L78"/>
+  <autoFilter ref="A1:L100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4139,7 +5057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4155,7 +5073,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-08</t>
+          <t>generated 2026-10-11</t>
         </is>
       </c>
     </row>
@@ -4166,7 +5084,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
@@ -4176,7 +5094,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -4186,7 +5104,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -4196,7 +5114,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -4214,7 +5132,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8-35</t>
+          <t>31-53</t>
         </is>
       </c>
     </row>
@@ -4325,7 +5243,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-08</t>
+          <t xml:space="preserve">  2026-10-11</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4334,253 +5252,6 @@
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-08</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>daily-20</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-12 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4987,66 +4987,123 @@
       <c r="L99" s="5" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="inlineStr">
+      <c r="A100" s="4" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>daily-20</t>
         </is>
       </c>
-      <c r="C100" s="7" t="inlineStr">
-        <is>
-          <t>Browns +2.5 (-110)
-Vikings -2.5 (+100)
-Under 46.5 (-118)
-Browns ML (+114)
-Over 43.5 (-108)
-Eagles +7.5 (+100)
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Browns +2.5 (-110) ✗
+Vikings -2.5 (+100) ✓
+Under 46.5 (-118) ✓
+Browns ML (+114) ✗
+Over 43.5 (-108) ✓
+Eagles +7.5 (+100) ✓
 Dolphins +7 (-110)
-Giants +3.5 (-108)
-Titans +7 (-112)
-Over 41.5 (-105)
-Over 54.5 (-105)
-Under 41.5 (-108)
-Under 43.5 (-112)
-Over 45.5 (-115)
-Under 43.5 (-110)
-Over 45.5 (-105)
-49ers +3 (-105)
-Chargers +3.5 (-112)
-Under 41.5 (-115)
-Colts +2.5 (+100)</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="n">
+Giants +3.5 (-108) ✓
+Titans +7 (-112) ✗
+Over 41.5 (-105) ✓
+Over 54.5 (-105) ✓
+Under 41.5 (-108) ✓
+Under 43.5 (-112) ✗
+Over 45.5 (-115) ✓
+Under 43.5 (-110) ✗
+Over 45.5 (-105) ✓
+49ers +3 (-105) ✓
+Chargers +3.5 (-112) ✗
+Under 41.5 (-115) ✓
+Colts +2.5 (+100) ✗</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="E100" s="6" t="inlineStr"/>
-      <c r="F100" s="6" t="inlineStr"/>
-      <c r="G100" s="6" t="inlineStr">
+      <c r="E100" s="4" t="inlineStr"/>
+      <c r="F100" s="4" t="inlineStr"/>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr"/>
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Leg record 12-7-1 excl push; staked (ranks 1-5) 3-2; CLV 1 beat / 3 lost / 15 push / 1 missing (ML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>Rays -1.5 (+130)
+Golden Knights ML (-102)
+Bills +3.5 (-118)
+Under 54.5 (-110)
+Rays ML (-172)
+Senators ML (+114)
+Brewers ML (+115)
+Under 6.5 (-110)
+Under 6 (-110)
+Under 5.5 (-110)
+Brewers +1.5 (-161)
+Bills ML (+148)
+Under 7 (-122)
+Under 6.5 (+101)</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E101" s="6" t="inlineStr"/>
+      <c r="F101" s="6" t="inlineStr"/>
+      <c r="G101" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H100" s="6" t="inlineStr"/>
-      <c r="I100" s="6" t="inlineStr">
+      <c r="H101" s="6" t="inlineStr"/>
+      <c r="I101" s="6" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="J100" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr"/>
-      <c r="L100" s="7" t="inlineStr"/>
+      <c r="J101" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr"/>
+      <c r="L101" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L100"/>
+  <autoFilter ref="A1:L101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5073,7 +5130,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-11</t>
+          <t>generated 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -5094,7 +5151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -5132,7 +5189,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>31-53</t>
+          <t>32-53</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5300,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-11</t>
+          <t xml:space="preserve">  2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-13 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5050,60 +5050,119 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>daily-20</t>
         </is>
       </c>
-      <c r="C101" s="7" t="inlineStr">
-        <is>
-          <t>Rays -1.5 (+130)
-Golden Knights ML (-102)
-Bills +3.5 (-118)
-Under 54.5 (-110)
-Rays ML (-172)
-Senators ML (+114)
-Brewers ML (+115)
-Under 6.5 (-110)
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Rays -1.5 (+130) ✗
+Golden Knights ML (-102) ✗
+Bills +3.5 (-118) ✓
+Under 54.5 (-110) ✓
+Rays ML (-172) ✗
+Senators ML (+114) ✓
+Brewers ML (+115) ✓
+Under 6.5 (-110) ✗
 Under 6 (-110)
-Under 5.5 (-110)
-Brewers +1.5 (-161)
-Bills ML (+148)
-Under 7 (-122)
-Under 6.5 (+101)</t>
-        </is>
-      </c>
-      <c r="D101" s="6" t="n">
+Under 5.5 (-110) ✓
+Brewers +1.5 (-161) ✓
+Bills ML (+148) ✓
+Under 7 (-122) ✗
+Under 6.5 (+101) ✗</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="E101" s="6" t="inlineStr"/>
-      <c r="F101" s="6" t="inlineStr"/>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="E101" s="4" t="inlineStr"/>
+      <c r="F101" s="4" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr"/>
+      <c r="L101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>Kraken ML (+101)
+Islanders ML (-218)
+Hurricanes ML (-158)
+Jets ML (-111)
+Rangers ML (+140)
+Predators ML (+109)
+Bruins ML (-104)
+Canadiens ML (-157)
+Blue Jackets ML (-123)
+Under 47.5 (-110)
+Penguins ML (-141)
+Guardians ML (+119)
+Lightning ML (-162)
+Under 6 (-110)
+Under 5.5 (+100)
+Over 6.5 (-105)
+Ducks ML (-205)
+Avalanche ML (-114)
+Under 6 (-110)
+Oilers ML (-125)</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E102" s="6" t="inlineStr"/>
+      <c r="F102" s="6" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H101" s="6" t="inlineStr"/>
-      <c r="I101" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings</t>
-        </is>
-      </c>
-      <c r="J101" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr"/>
-      <c r="L101" s="7" t="inlineStr"/>
+      <c r="H102" s="6" t="inlineStr"/>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>consensus (wunderdog)</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
+      <c r="L102" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L101"/>
+  <autoFilter ref="A1:L102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5130,7 +5189,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-12</t>
+          <t>generated 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5200,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -5151,7 +5210,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -5189,7 +5248,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>32-53</t>
+          <t>33-53</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5359,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-12</t>
+          <t xml:space="preserve">  2026-10-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-14 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5103,66 +5103,119 @@
       <c r="L101" s="5" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="6" t="inlineStr">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>daily-20</t>
         </is>
       </c>
-      <c r="C102" s="7" t="inlineStr">
-        <is>
-          <t>Kraken ML (+101)
-Islanders ML (-218)
-Hurricanes ML (-158)
-Jets ML (-111)
-Rangers ML (+140)
-Predators ML (+109)
-Bruins ML (-104)
-Canadiens ML (-157)
-Blue Jackets ML (-123)
-Under 47.5 (-110)
-Penguins ML (-141)
-Guardians ML (+119)
-Lightning ML (-162)
-Under 6 (-110)
-Under 5.5 (+100)
-Over 6.5 (-105)
-Ducks ML (-205)
-Avalanche ML (-114)
-Under 6 (-110)
-Oilers ML (-125)</t>
-        </is>
-      </c>
-      <c r="D102" s="6" t="n">
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Kraken ML (+101) ✓
+Islanders ML (-218) ✓
+Hurricanes ML (-158) ✓
+Jets ML (-111) ✓
+Rangers ML (+140) ✓
+Predators ML (+109) ✗
+Bruins ML (-104) ✓
+Canadiens ML (-157) ✓
+Blue Jackets ML (-123) ✗
+Under 47.5 (-110) ✗
+Penguins ML (-141) ✗
+Guardians ML (+119) ✗
+Lightning ML (-162) ✗
+Under 6 (-110) ✓
+Under 5.5 (+100) ✗
+Over 6.5 (-105) ✓
+Ducks ML (-205) ✗
+Avalanche ML (-114) ✓
+Under 6 (-110) ✗
+Oilers ML (-125) ✓</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="E102" s="6" t="inlineStr"/>
-      <c r="F102" s="6" t="inlineStr"/>
-      <c r="G102" s="6" t="inlineStr">
+      <c r="E102" s="4" t="inlineStr"/>
+      <c r="F102" s="4" t="inlineStr"/>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr"/>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>consensus (wunderdog)</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr"/>
+      <c r="L102" s="5" t="inlineStr">
+        <is>
+          <t>Legs 11-9: staked set 1-0 (SEA ML +101 cashed in SO). Frozen Frenzy night: dogs mostly barked (Rangers +140, Kraken +101 both won). CLV: 1 beat (CLE +119 vs near-close +114), 19 inevaluable - no verifiable NHL closings v</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>daily-20</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>Sam Houston +1.5 (-105)
+Bearkats ML (+105)
+Kennesaw State -3 (-112)
+Under 6.5 (-105)
+Under 5.5 (+110)
+Stars ML (+120)
+Brewers ML (+162)
+Under 52.5 (-105)
+Under 52.5 (-110)
+Under 7.5 (-112)</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E103" s="6" t="inlineStr"/>
+      <c r="F103" s="6" t="inlineStr"/>
+      <c r="G103" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H102" s="6" t="inlineStr"/>
-      <c r="I102" s="6" t="inlineStr">
-        <is>
-          <t>consensus (wunderdog)</t>
-        </is>
-      </c>
-      <c r="J102" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr"/>
-      <c r="L102" s="7" t="inlineStr"/>
+      <c r="H103" s="6" t="inlineStr"/>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J103" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K103" s="6" t="inlineStr"/>
+      <c r="L103" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L102"/>
+  <autoFilter ref="A1:L103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5189,7 +5242,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-13</t>
+          <t>generated 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5253,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -5210,7 +5263,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -5248,7 +5301,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>33-53</t>
+          <t>34-53</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5412,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-13</t>
+          <t xml:space="preserve">  2026-10-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-15 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5166,56 +5166,98 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="6" t="inlineStr">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B103" s="6" t="inlineStr">
+      <c r="B103" s="2" t="inlineStr">
         <is>
           <t>daily-20</t>
         </is>
       </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>Sam Houston +1.5 (-105)
-Bearkats ML (+105)
-Kennesaw State -3 (-112)
-Under 6.5 (-105)
-Under 5.5 (+110)
-Stars ML (+120)
-Brewers ML (+162)
-Under 52.5 (-105)
-Under 52.5 (-110)
-Under 7.5 (-112)</t>
-        </is>
-      </c>
-      <c r="D103" s="6" t="n">
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Sam Houston +1.5 (-105) ✗
+Bearkats ML (+105) ✗
+Kennesaw State -3 (-112) ✗
+Under 6.5 (-105) ✗
+Under 5.5 (+110) ✓
+Stars ML (+120) ✓
+Brewers ML (+162) ✓
+Under 52.5 (-105) ✓
+Under 52.5 (-110) ✓
+Under 7.5 (-112) ✗</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E103" s="6" t="inlineStr"/>
-      <c r="F103" s="6" t="inlineStr"/>
-      <c r="G103" s="6" t="inlineStr">
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>Rangers ML (+124)
+East Carolina -4.5 (-110)
+Under 6.5 (+100)</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E104" s="6" t="inlineStr"/>
+      <c r="F104" s="6" t="inlineStr"/>
+      <c r="G104" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H103" s="6" t="inlineStr"/>
-      <c r="I103" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings</t>
-        </is>
-      </c>
-      <c r="J103" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K103" s="6" t="inlineStr"/>
-      <c r="L103" s="7" t="inlineStr"/>
+      <c r="H104" s="6" t="inlineStr"/>
+      <c r="I104" s="6" t="inlineStr">
+        <is>
+          <t>DraftKings (via scoresandstats DK read; +120 consensus)</t>
+        </is>
+      </c>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K104" s="6" t="inlineStr"/>
+      <c r="L104" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L103"/>
+  <autoFilter ref="A1:L104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5242,7 +5284,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-14</t>
+          <t>generated 2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5295,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
@@ -5273,7 +5315,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -5301,7 +5343,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>34-53</t>
+          <t>34-54</t>
         </is>
       </c>
     </row>
@@ -5412,12 +5454,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-14</t>
+          <t xml:space="preserve">  2026-10-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>daily-20</t>
+          <t>uncapped</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-16 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5215,49 +5215,90 @@
       <c r="L103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="B104" s="6" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C104" s="7" t="inlineStr">
-        <is>
-          <t>Rangers ML (+124)
-East Carolina -4.5 (-110)
-Under 6.5 (+100)</t>
-        </is>
-      </c>
-      <c r="D104" s="6" t="n">
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Rangers ML (+124) ✗
+East Carolina -4.5 (-110) ✗
+Under 6.5 (+100) ✓</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E104" s="6" t="inlineStr"/>
-      <c r="F104" s="6" t="inlineStr"/>
-      <c r="G104" s="6" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings (via scoresandstats DK read; +120 consensus)</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>Memphis -7 (-110)
+Under 6.5 (-110)</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E105" s="6" t="inlineStr"/>
+      <c r="F105" s="6" t="inlineStr"/>
+      <c r="G105" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H104" s="6" t="inlineStr"/>
-      <c r="I104" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings (via scoresandstats DK read; +120 consensus)</t>
-        </is>
-      </c>
-      <c r="J104" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K104" s="6" t="inlineStr"/>
-      <c r="L104" s="7" t="inlineStr"/>
+      <c r="H105" s="6" t="inlineStr"/>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>DraftKings (via SBR DK read; -7 -105 to -110 market)</t>
+        </is>
+      </c>
+      <c r="J105" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K105" s="6" t="inlineStr"/>
+      <c r="L105" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L104"/>
+  <autoFilter ref="A1:L105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5284,7 +5325,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-15</t>
+          <t>generated 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5336,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4">
@@ -5315,7 +5356,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -5343,7 +5384,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>34-54</t>
+          <t>34-55</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5495,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-15</t>
+          <t xml:space="preserve">  2026-10-16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-17 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>Memphis -7 (-110)
+          <t>Memphis -7 (-110) ✗
 Under 6.5 (-110)</t>
         </is>
       </c>
@@ -5297,8 +5297,48 @@
       <c r="K105" s="6" t="inlineStr"/>
       <c r="L105" s="7" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>Bruins ML (+112)</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="6" t="inlineStr"/>
+      <c r="F106" s="6" t="inlineStr"/>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr"/>
+      <c r="I106" s="6" t="inlineStr">
+        <is>
+          <t>FanDuel (DK price unverified)</t>
+        </is>
+      </c>
+      <c r="J106" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K106" s="6" t="inlineStr"/>
+      <c r="L106" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L105"/>
+  <autoFilter ref="A1:L106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5309,7 +5349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5325,7 +5365,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-16</t>
+          <t>generated 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5376,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4">
@@ -5366,7 +5406,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -5504,6 +5544,19 @@
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026-10-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-18 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5257,88 +5257,137 @@
       <c r="L104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="6" t="inlineStr">
+      <c r="A105" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C105" s="7" t="inlineStr">
+      <c r="C105" s="3" t="inlineStr">
         <is>
           <t>Memphis -7 (-110) ✗
-Under 6.5 (-110)</t>
-        </is>
-      </c>
-      <c r="D105" s="6" t="n">
+Under 6.5 (-110) ✗</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E105" s="6" t="inlineStr"/>
-      <c r="F105" s="6" t="inlineStr"/>
-      <c r="G105" s="6" t="inlineStr">
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings (via SBR DK read; -7 -105 to -110 market)</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>Card 0-2: Memphis -7 lost 31-17 (10/16), TB@CLE G4 Under 6.5 lost 7-3 (10/17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Bruins ML (+112) ✓</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="4" t="inlineStr"/>
+      <c r="F106" s="4" t="inlineStr"/>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr"/>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>FanDuel +112 logged; DK verified +114 (pregame sweep)</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K106" s="4" t="inlineStr"/>
+      <c r="L106" s="5" t="inlineStr">
+        <is>
+          <t>Card 1-0: Bruins ML won 4-1 (10/17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>Under 41.5 (-110)
+Under 39.5 (-110)</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E107" s="6" t="inlineStr"/>
+      <c r="F107" s="6" t="inlineStr"/>
+      <c r="G107" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H105" s="6" t="inlineStr"/>
-      <c r="I105" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings (via SBR DK read; -7 -105 to -110 market)</t>
-        </is>
-      </c>
-      <c r="J105" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K105" s="6" t="inlineStr"/>
-      <c r="L105" s="7" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>uncapped</t>
-        </is>
-      </c>
-      <c r="C106" s="7" t="inlineStr">
-        <is>
-          <t>Bruins ML (+112)</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" s="6" t="inlineStr"/>
-      <c r="F106" s="6" t="inlineStr"/>
-      <c r="G106" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H106" s="6" t="inlineStr"/>
-      <c r="I106" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (DK price unverified)</t>
-        </is>
-      </c>
-      <c r="J106" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K106" s="6" t="inlineStr"/>
-      <c r="L106" s="7" t="inlineStr"/>
+      <c r="H107" s="6" t="inlineStr"/>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J107" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K107" s="6" t="inlineStr"/>
+      <c r="L107" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L106"/>
+  <autoFilter ref="A1:L107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5349,7 +5398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5365,7 +5414,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-17</t>
+          <t>generated 2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5425,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -5386,7 +5435,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -5396,7 +5445,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -5406,7 +5455,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -5424,7 +5473,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>34-55</t>
+          <t>35-56</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5584,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-16</t>
+          <t xml:space="preserve">  2026-10-18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5544,19 +5593,6 @@
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-17</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>uncapped</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-19 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5346,48 +5346,88 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="6" t="inlineStr">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="B107" s="6" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>Under 41.5 (-110)
-Under 39.5 (-110)</t>
-        </is>
-      </c>
-      <c r="D107" s="6" t="n">
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Under 41.5 (-110) ✓
+Under 39.5 (-110) ✓</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E107" s="6" t="inlineStr"/>
-      <c r="F107" s="6" t="inlineStr"/>
-      <c r="G107" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="H107" s="6" t="inlineStr"/>
-      <c r="I107" s="6" t="inlineStr">
+      <c r="E107" s="4" t="inlineStr"/>
+      <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr"/>
+      <c r="I107" s="4" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="J107" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K107" s="6" t="inlineStr"/>
-      <c r="L107" s="7" t="inlineStr"/>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr"/>
+      <c r="L107" s="5" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Over 53.5 (-110) ✗</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings (Over seen -105 to -112; confirm live)</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L107"/>
+  <autoFilter ref="A1:L108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5398,7 +5438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5414,7 +5454,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-18</t>
+          <t>generated 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
@@ -5435,7 +5475,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -5445,7 +5485,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -5455,7 +5495,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -5473,7 +5513,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>35-56</t>
+          <t>36-57</t>
         </is>
       </c>
     </row>
@@ -5580,19 +5620,6 @@
           <t>+196</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026-10-18</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>uncapped</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-20 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5426,8 +5426,89 @@
       <c r="K108" s="2" t="inlineStr"/>
       <c r="L108" s="3" t="inlineStr"/>
     </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>49ers -7.5 (-110) ✗</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr"/>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings (seen -108 to -110; confirm live)</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>Under 45.5 (-110)
+South Alabama -3 (-112)</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E110" s="6" t="inlineStr"/>
+      <c r="F110" s="6" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr"/>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr"/>
+      <c r="L110" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L108"/>
+  <autoFilter ref="A1:L110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5438,7 +5519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5454,7 +5535,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-19</t>
+          <t>generated 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -5465,7 +5546,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4">
@@ -5485,7 +5566,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -5495,7 +5576,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -5513,7 +5594,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-57</t>
+          <t>36-58</t>
         </is>
       </c>
     </row>
@@ -5620,6 +5701,19 @@
           <t>+196</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026-10-20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-21 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5467,48 +5467,91 @@
       <c r="L109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C110" s="7" t="inlineStr">
-        <is>
-          <t>Under 45.5 (-110)
-South Alabama -3 (-112)</t>
-        </is>
-      </c>
-      <c r="D110" s="6" t="n">
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Under 45.5 (-110) ✗
+South Alabama -3 (-112) ✗</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E110" s="6" t="inlineStr"/>
-      <c r="F110" s="6" t="inlineStr"/>
-      <c r="G110" s="6" t="inlineStr">
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>DraftKings</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>Sam Houston State +2.5 (-110)
+New Orleans Pelicans ML (+130)
+Phoenix Suns ML (+120)
+Ottawa Senators ML (-108)</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E111" s="6" t="inlineStr"/>
+      <c r="F111" s="6" t="inlineStr"/>
+      <c r="G111" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H110" s="6" t="inlineStr"/>
-      <c r="I110" s="6" t="inlineStr">
-        <is>
-          <t>DraftKings</t>
-        </is>
-      </c>
-      <c r="J110" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K110" s="6" t="inlineStr"/>
-      <c r="L110" s="7" t="inlineStr"/>
+      <c r="H111" s="6" t="inlineStr"/>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>consensus (DK price not isolated; bet365 early had NMSU -2.5 -120)</t>
+        </is>
+      </c>
+      <c r="J111" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K111" s="6" t="inlineStr"/>
+      <c r="L111" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L110"/>
+  <autoFilter ref="A1:L111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5535,7 +5578,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-20</t>
+          <t>generated 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5546,7 +5589,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -5566,7 +5609,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -5594,7 +5637,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-58</t>
+          <t>36-59</t>
         </is>
       </c>
     </row>
@@ -5705,7 +5748,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-20</t>
+          <t xml:space="preserve">  2026-10-21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-22 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5508,50 +5508,98 @@
       <c r="L110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="6" t="inlineStr">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B111" s="6" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C111" s="7" t="inlineStr">
-        <is>
-          <t>Sam Houston State +2.5 (-110)
-New Orleans Pelicans ML (+130)
-Phoenix Suns ML (+120)
-Ottawa Senators ML (-108)</t>
-        </is>
-      </c>
-      <c r="D111" s="6" t="n">
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Sam Houston State +2.5 (-110) ✗
+New Orleans Pelicans ML (+130) ✗
+Phoenix Suns ML (+120) ✗
+Ottawa Senators ML (-108) ✓</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E111" s="6" t="inlineStr"/>
-      <c r="F111" s="6" t="inlineStr"/>
-      <c r="G111" s="6" t="inlineStr">
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr"/>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr"/>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>consensus (DK price not isolated; bet365 early had NMSU -2.5 -120)</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr">
+        <is>
+          <t>Card 1-3: only Senators ML won (5-1). Staked set 1-1 (SHSU +2.5 loss, OTT ML win). Ullmark left 3rd period with lower-body strain, re-evaluated Thursday — watch for tonight's Sharks@Senators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>Senators ML (-128)
+Penguins ML (-115)
+Islanders ML (-115)
+Cavaliers ML (+124)
+Bruins ML (-160)</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E112" s="6" t="inlineStr"/>
+      <c r="F112" s="6" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H111" s="6" t="inlineStr"/>
-      <c r="I111" s="6" t="inlineStr">
-        <is>
-          <t>consensus (DK price not isolated; bet365 early had NMSU -2.5 -120)</t>
-        </is>
-      </c>
-      <c r="J111" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K111" s="6" t="inlineStr"/>
-      <c r="L111" s="7" t="inlineStr"/>
+      <c r="H112" s="6" t="inlineStr"/>
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>consensus (no DK line found; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J112" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K112" s="6" t="inlineStr"/>
+      <c r="L112" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L111"/>
+  <autoFilter ref="A1:L112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5578,7 +5626,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-21</t>
+          <t>generated 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5589,7 +5637,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -5609,7 +5657,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6">
@@ -5637,7 +5685,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-59</t>
+          <t>36-60</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5796,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-21</t>
+          <t xml:space="preserve">  2026-10-22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-23 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -5567,11 +5567,11 @@
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>Senators ML (-128)
-Penguins ML (-115)
-Islanders ML (-115)
-Cavaliers ML (+124)
-Bruins ML (-160)</t>
+          <t>Senators ML (-128) ✗
+Penguins ML (-115) ✓
+Islanders ML (-115) ✗
+Cavaliers ML (+124) ✗
+Bruins ML (-160) ✓</t>
         </is>
       </c>
       <c r="D112" s="6" t="n">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-22</t>
+          <t>generated 2026-10-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily sync: 2026-10-24 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5598,8 +5598,52 @@
       <c r="K112" s="6" t="inlineStr"/>
       <c r="L112" s="7" t="inlineStr"/>
     </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets ML (+130)
+Tennessee +2.5 (-112)
+Chicago Bulls ML (-104)
+Buffalo Sabres ML (+106)
+Under 6.5 (-106)</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E113" s="6" t="inlineStr"/>
+      <c r="F113" s="6" t="inlineStr"/>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="inlineStr"/>
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>FanDuel +130 (DK price not isolated; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J113" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K113" s="6" t="inlineStr"/>
+      <c r="L113" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L112"/>
+  <autoFilter ref="A1:L113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5610,7 +5654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5626,7 +5670,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-23</t>
+          <t>generated 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5681,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -5667,7 +5711,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -5805,6 +5849,19 @@
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026-10-24</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-25 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5599,51 +5599,104 @@
       <c r="L112" s="7" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="6" t="inlineStr">
+      <c r="A113" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="B113" s="6" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C113" s="7" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets ML (+130)
-Tennessee +2.5 (-112)
-Chicago Bulls ML (-104)
-Buffalo Sabres ML (+106)
-Under 6.5 (-106)</t>
-        </is>
-      </c>
-      <c r="D113" s="6" t="n">
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets ML (+130) ✓
+Tennessee +2.5 (-112) ✗
+Chicago Bulls ML (-104) ✗
+Buffalo Sabres ML (+106) ✗
+Under 6.5 (-106) ✗</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E113" s="6" t="inlineStr"/>
-      <c r="F113" s="6" t="inlineStr"/>
-      <c r="G113" s="6" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr"/>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel +130 (DK price not isolated; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>Card 1-4: only Hornets ML won (115-110). Staked set 0-3 (Tennessee +2.5 lost by half a point, 27-24 on a 48-yd FG as time expired; Sabres ML lost 4-3 OT; WS G2 Under 6.5 lost, total 9). NBA paper legs 1-1 (Hornets W, Bul</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens +1.5 (-105)
+Carolina Panthers ML (-155)
+Pittsburgh Steelers ML (-162)
+Kansas City Chiefs +3 (-110)
+Detroit Pistons ML (+122)
+Minnesota Timberwolves ML (-108)
+Winnipeg Jets ML (+107)
+Nashville Predators ML (+188)
+New York Islanders +1.5 (-158)
+Chicago Blackhawks ML (+150)</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E114" s="6" t="inlineStr"/>
+      <c r="F114" s="6" t="inlineStr"/>
+      <c r="G114" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H113" s="6" t="inlineStr"/>
-      <c r="I113" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel +130 (DK price not isolated; verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J113" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K113" s="6" t="inlineStr"/>
-      <c r="L113" s="7" t="inlineStr"/>
+      <c r="H114" s="6" t="inlineStr"/>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>consensus (LineTerminal; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J114" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K114" s="6" t="inlineStr"/>
+      <c r="L114" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L113"/>
+  <autoFilter ref="A1:L114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5670,7 +5723,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-24</t>
+          <t>generated 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5681,7 +5734,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -5701,7 +5754,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
@@ -5729,7 +5782,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-60</t>
+          <t>36-61</t>
         </is>
       </c>
     </row>
@@ -5853,7 +5906,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-24</t>
+          <t xml:space="preserve">  2026-10-25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-26 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5647,56 +5647,97 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="6" t="inlineStr">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C114" s="7" t="inlineStr">
-        <is>
-          <t>Baltimore Ravens +1.5 (-105)
-Carolina Panthers ML (-155)
-Pittsburgh Steelers ML (-162)
-Kansas City Chiefs +3 (-110)
-Detroit Pistons ML (+122)
-Minnesota Timberwolves ML (-108)
-Winnipeg Jets ML (+107)
-Nashville Predators ML (+188)
-New York Islanders +1.5 (-158)
-Chicago Blackhawks ML (+150)</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="n">
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens +1.5 (-105) ✗
+Carolina Panthers ML (-155) ✗
+Pittsburgh Steelers ML (-162) ✓
+Kansas City Chiefs +3 (-110) ✗
+Detroit Pistons ML (+122) ✓
+Minnesota Timberwolves ML (-108) ✓
+Winnipeg Jets ML (+107) ✗
+Nashville Predators ML (+188) ✓
+New York Islanders +1.5 (-158) ✗
+Chicago Blackhawks ML (+150) ✗</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E114" s="6" t="inlineStr"/>
-      <c r="F114" s="6" t="inlineStr"/>
-      <c r="G114" s="6" t="inlineStr">
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>consensus (LineTerminal; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>New York Rangers ML (-126)
+Calgary Flames ML (+136)</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E115" s="6" t="inlineStr"/>
+      <c r="F115" s="6" t="inlineStr"/>
+      <c r="G115" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H114" s="6" t="inlineStr"/>
-      <c r="I114" s="6" t="inlineStr">
-        <is>
-          <t>consensus (LineTerminal; verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J114" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K114" s="6" t="inlineStr"/>
-      <c r="L114" s="7" t="inlineStr"/>
+      <c r="H115" s="6" t="inlineStr"/>
+      <c r="I115" s="6" t="inlineStr">
+        <is>
+          <t>FanDuel</t>
+        </is>
+      </c>
+      <c r="J115" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K115" s="6" t="inlineStr"/>
+      <c r="L115" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L114"/>
+  <autoFilter ref="A1:L115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5723,7 +5764,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-25</t>
+          <t>generated 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5734,7 +5775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4">
@@ -5754,7 +5795,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6">
@@ -5782,7 +5823,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-61</t>
+          <t>36-62</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5947,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-25</t>
+          <t xml:space="preserve">  2026-10-26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-27 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5708,8 +5708,8 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>New York Rangers ML (-126)
-Calgary Flames ML (+136)</t>
+          <t>New York Rangers ML (-126) ✗
+Calgary Flames ML (+136) ✓</t>
         </is>
       </c>
       <c r="D115" s="6" t="n">
@@ -5734,10 +5734,55 @@
         </is>
       </c>
       <c r="K115" s="6" t="inlineStr"/>
-      <c r="L115" s="7" t="inlineStr"/>
+      <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t>10/26 card 1-1 (staked 1-1): NYR ML LOSS 6-3, CGY ML WIN 5-2. CLV: 1 beat (NYR), 1 push (CGY) - no staked leg missing a close, so the 10/26 CLV gate is clear for today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>Dallas Stars ML (-125)
+Los Angeles Lakers ML (-142)</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E116" s="6" t="inlineStr"/>
+      <c r="F116" s="6" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr"/>
+      <c r="I116" s="6" t="inlineStr">
+        <is>
+          <t>FanDuel (DK price not found; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J116" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K116" s="6" t="inlineStr"/>
+      <c r="L116" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L115"/>
+  <autoFilter ref="A1:L116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5748,7 +5793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5764,7 +5809,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-26</t>
+          <t>generated 2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5820,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
@@ -5805,7 +5850,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -5956,6 +6001,19 @@
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026-10-27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily sync: 2026-10-28 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5741,48 +5741,92 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="6" t="inlineStr">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C116" s="7" t="inlineStr">
-        <is>
-          <t>Dallas Stars ML (-125)
-Los Angeles Lakers ML (-142)</t>
-        </is>
-      </c>
-      <c r="D116" s="6" t="n">
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Dallas Stars ML (-125) ✗
+Los Angeles Lakers ML (-142) ✗</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E116" s="6" t="inlineStr"/>
-      <c r="F116" s="6" t="inlineStr"/>
-      <c r="G116" s="6" t="inlineStr">
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (DK price not found; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves ML (-152)
+Oklahoma City Thunder ML (-225)
+Seattle Kraken ML (+102)
+Colorado Avalanche ML (-178)
+Cleveland Cavaliers ML (-375)</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E117" s="6" t="inlineStr"/>
+      <c r="F117" s="6" t="inlineStr"/>
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H116" s="6" t="inlineStr"/>
-      <c r="I116" s="6" t="inlineStr">
+      <c r="H117" s="6" t="inlineStr"/>
+      <c r="I117" s="6" t="inlineStr">
         <is>
           <t>FanDuel (DK price not found; verify in DK app)</t>
         </is>
       </c>
-      <c r="J116" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K116" s="6" t="inlineStr"/>
-      <c r="L116" s="7" t="inlineStr"/>
+      <c r="J117" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K117" s="6" t="inlineStr"/>
+      <c r="L117" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L116"/>
+  <autoFilter ref="A1:L117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5809,7 +5853,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-27</t>
+          <t>generated 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5864,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
@@ -5840,7 +5884,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -5868,7 +5912,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-62</t>
+          <t>36-63</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6049,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-27</t>
+          <t xml:space="preserve">  2026-10-28</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-29 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5782,51 +5782,95 @@
       <c r="L116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="6" t="inlineStr">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="B117" s="6" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C117" s="7" t="inlineStr">
-        <is>
-          <t>Minnesota Timberwolves ML (-152)
-Oklahoma City Thunder ML (-225)
-Seattle Kraken ML (+102)
-Colorado Avalanche ML (-178)
-Cleveland Cavaliers ML (-375)</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="n">
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves ML (-152) ✗
+Oklahoma City Thunder ML (-225) ✗
+Seattle Kraken ML (+102) ✓
+Colorado Avalanche ML (-178) ✓
+Cleveland Cavaliers ML (-375) ✓</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E117" s="6" t="inlineStr"/>
-      <c r="F117" s="6" t="inlineStr"/>
-      <c r="G117" s="6" t="inlineStr">
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr"/>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (DK price not found; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>Scored 2026-10-29: 3-2 (SEA ML W 5-4, COL ML W 5-2, CLE ML W 121-111; MIN ML L 114-119, OKC ML L 96-120). All paper-only (no NFL on slate, NFL-only staking rule). Closing odds not captured — flagged as missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B118" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>Pittsburgh Penguins ML (+114)</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="6" t="inlineStr"/>
+      <c r="F118" s="6" t="inlineStr"/>
+      <c r="G118" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H117" s="6" t="inlineStr"/>
-      <c r="I117" s="6" t="inlineStr">
+      <c r="H118" s="6" t="inlineStr"/>
+      <c r="I118" s="6" t="inlineStr">
         <is>
           <t>FanDuel (DK price not found; verify in DK app)</t>
         </is>
       </c>
-      <c r="J117" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K117" s="6" t="inlineStr"/>
-      <c r="L117" s="7" t="inlineStr"/>
+      <c r="J118" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K118" s="6" t="inlineStr"/>
+      <c r="L118" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L117"/>
+  <autoFilter ref="A1:L118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5853,7 +5897,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-28</t>
+          <t>generated 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5908,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
@@ -5884,7 +5928,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
@@ -5912,7 +5956,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-63</t>
+          <t>36-64</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6093,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-28</t>
+          <t xml:space="preserve">  2026-10-29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-30 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5830,47 +5830,93 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="6" t="inlineStr">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="B118" s="6" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C118" s="7" t="inlineStr">
-        <is>
-          <t>Pittsburgh Penguins ML (+114)</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="n">
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Pittsburgh Penguins ML (+114) ✗</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E118" s="6" t="inlineStr"/>
-      <c r="F118" s="6" t="inlineStr"/>
-      <c r="G118" s="6" t="inlineStr">
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel (DK price not found; verify in DK app)</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets ML (+102)
+Phoenix Suns ML (+154)
+Miami Heat ML (-300)
+Detroit Pistons ML (-295)
+Houston Rockets ML (-215)
+Vegas Golden Knights ML (-113)
+Tulane Green Wave ML (-345)</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E119" s="6" t="inlineStr"/>
+      <c r="F119" s="6" t="inlineStr"/>
+      <c r="G119" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H118" s="6" t="inlineStr"/>
-      <c r="I118" s="6" t="inlineStr">
-        <is>
-          <t>FanDuel (DK price not found; verify in DK app)</t>
-        </is>
-      </c>
-      <c r="J118" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K118" s="6" t="inlineStr"/>
-      <c r="L118" s="7" t="inlineStr"/>
+      <c r="H119" s="6" t="inlineStr"/>
+      <c r="I119" s="6" t="inlineStr">
+        <is>
+          <t>FanDuel</t>
+        </is>
+      </c>
+      <c r="J119" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K119" s="6" t="inlineStr"/>
+      <c r="L119" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L118"/>
+  <autoFilter ref="A1:L119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5897,7 +5943,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-29</t>
+          <t>generated 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5954,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4">
@@ -5928,7 +5974,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
@@ -5956,7 +6002,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-64</t>
+          <t>36-65</t>
         </is>
       </c>
     </row>
@@ -6093,7 +6139,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-29</t>
+          <t xml:space="preserve">  2026-10-30</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>

<commit_message>
Daily sync: 2026-10-31 (ledgers, dashboard data)
</commit_message>
<xml_diff>
--- a/data/bet-matrix.xlsx
+++ b/data/bet-matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$L$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5870,53 +5870,110 @@
       <c r="L118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="6" t="inlineStr">
+      <c r="A119" s="2" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="B119" s="6" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>uncapped</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets ML (+102)
-Phoenix Suns ML (+154)
-Miami Heat ML (-300)
-Detroit Pistons ML (-295)
-Houston Rockets ML (-215)
-Vegas Golden Knights ML (-113)
-Tulane Green Wave ML (-345)</t>
-        </is>
-      </c>
-      <c r="D119" s="6" t="n">
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets ML (+102) ✗
+Phoenix Suns ML (+154) ✗
+Miami Heat ML (-300) ✓
+Detroit Pistons ML (-295) ✓
+Houston Rockets ML (-215) ✗
+Vegas Golden Knights ML (-113) ✗
+Tulane Green Wave ML (-345) ✓</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E119" s="6" t="inlineStr"/>
-      <c r="F119" s="6" t="inlineStr"/>
-      <c r="G119" s="6" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr"/>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr"/>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>FanDuel</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B120" s="6" t="inlineStr">
+        <is>
+          <t>uncapped</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder ML (+146)
+San Diego State ML (-132)
+Boston Bruins ML (-220)
+Colorado State ML (+190)
+Fresno State ML (+185)
+Sacramento Kings ML (+370)
+South Florida ML (-310)
+Illinois ML (-135)
+Iowa ML (-135)
+Appalachian State ML (+180)
+Virginia ML (+390)
+Ottawa Senators ML (-134)
+Buffalo Sabres ML (-122)
+Tampa Bay Lightning ML (-166)
+Montreal Canadiens ML (-150)
+Philadelphia 76ers ML (-120)
+Clemson ML (+180)
+South Carolina ML (+142)</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E120" s="6" t="inlineStr"/>
+      <c r="F120" s="6" t="inlineStr"/>
+      <c r="G120" s="6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="H119" s="6" t="inlineStr"/>
-      <c r="I119" s="6" t="inlineStr">
+      <c r="H120" s="6" t="inlineStr"/>
+      <c r="I120" s="6" t="inlineStr">
         <is>
           <t>FanDuel</t>
         </is>
       </c>
-      <c r="J119" s="6" t="inlineStr">
-        <is>
-          <t>muse</t>
-        </is>
-      </c>
-      <c r="K119" s="6" t="inlineStr"/>
-      <c r="L119" s="7" t="inlineStr"/>
+      <c r="J120" s="6" t="inlineStr">
+        <is>
+          <t>muse</t>
+        </is>
+      </c>
+      <c r="K120" s="6" t="inlineStr"/>
+      <c r="L120" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L119"/>
+  <autoFilter ref="A1:L120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5943,7 +6000,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>generated 2026-10-30</t>
+          <t>generated 2026-10-31</t>
         </is>
       </c>
     </row>
@@ -5954,7 +6011,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4">
@@ -5974,7 +6031,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6">
@@ -6002,7 +6059,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36-65</t>
+          <t>36-66</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6196,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026-10-30</t>
+          <t xml:space="preserve">  2026-10-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>